<commit_message>
feat(parser): add support for Processus Excel format and Vis.js enhancements
- Added support in ExcelParserService for Processus, Sous-processus, Activité, Applications, and Composants columns
- Added multi-sheet sample Excel file with Processus & Activités sheet
- Added unit tests for Processus Excel format in ExcelParserServiceTest
- Added Vis.js layout switching, smart search focus, protocol edge filtering, fullscreen, and context menu
</commit_message>
<xml_diff>
--- a/src/main/resources/static/sample-flows.xlsx
+++ b/src/main/resources/static/sample-flows.xlsx
@@ -7,12 +7,13 @@
   </bookViews>
   <sheets>
     <sheet name="Flux_Applicatifs" r:id="rId3" sheetId="1"/>
+    <sheet name="Processus_et_Activités" r:id="rId4" sheetId="2"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="43">
   <si>
     <t>Source</t>
   </si>
@@ -78,6 +79,69 @@
   </si>
   <si>
     <t>JDBC Driver</t>
+  </si>
+  <si>
+    <t>Processus</t>
+  </si>
+  <si>
+    <t>Sous-processus</t>
+  </si>
+  <si>
+    <t>Activité</t>
+  </si>
+  <si>
+    <t>Applications</t>
+  </si>
+  <si>
+    <t>Composants</t>
+  </si>
+  <si>
+    <t>Ventes &amp; Commandes</t>
+  </si>
+  <si>
+    <t>Prise de commande</t>
+  </si>
+  <si>
+    <t>Saisie panier</t>
+  </si>
+  <si>
+    <t>Angular Frontend</t>
+  </si>
+  <si>
+    <t>Validation paiement</t>
+  </si>
+  <si>
+    <t>Stripe API</t>
+  </si>
+  <si>
+    <t>Gestion de stock</t>
+  </si>
+  <si>
+    <t>Réservation article</t>
+  </si>
+  <si>
+    <t>Spring Boot Service</t>
+  </si>
+  <si>
+    <t>Mise à jour stock</t>
+  </si>
+  <si>
+    <t>SQL Database</t>
+  </si>
+  <si>
+    <t>Support Client</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Traiter réclamation</t>
+  </si>
+  <si>
+    <t>CRM Application</t>
+  </si>
+  <si>
+    <t>Salesforce Module</t>
   </si>
 </sst>
 </file>
@@ -226,4 +290,116 @@
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="D1" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="E1" t="s" s="0">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
 </file>
</xml_diff>